<commit_message>
#186 oneshot support (take 2)
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carl\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D739A03-C40E-4E83-9007-7C2AB6857697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706EE84C-66AB-4422-A26D-B8FB4C52FBF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11070" yWindow="1260" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -26,14 +26,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>target</t>
   </si>
   <si>
-    <t>current unpadded</t>
-  </si>
-  <si>
     <t>save total</t>
   </si>
   <si>
@@ -50,16 +47,46 @@
   </si>
   <si>
     <t>delta</t>
+  </si>
+  <si>
+    <t>adding oneshot support</t>
+  </si>
+  <si>
+    <t>presquishdelta</t>
+  </si>
+  <si>
+    <t>unpadded squished</t>
+  </si>
+  <si>
+    <t>track flags vs serialization</t>
+  </si>
+  <si>
+    <t>base</t>
+  </si>
+  <si>
+    <t>oneshots on percussion tracks</t>
+  </si>
+  <si>
+    <t>fixed velocity on riser + snare tracks</t>
+  </si>
+  <si>
+    <t>uncompressed song data</t>
+  </si>
+  <si>
+    <t>compressed</t>
+  </si>
+  <si>
+    <t>both</t>
+  </si>
+  <si>
+    <t>with oneshot song payload</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0_ ;[Red]\-0\ "/>
-  </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -70,13 +97,6 @@
     <font>
       <sz val="8"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -102,10 +122,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -420,36 +439,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -462,7 +481,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
-        <f>E3-$Q$2</f>
+        <f>D3-$Q$2</f>
         <v>9328</v>
       </c>
       <c r="B3" s="1" t="str">
@@ -472,16 +491,16 @@
       <c r="C3">
         <v>117248</v>
       </c>
-      <c r="E3">
+      <c r="D3">
         <v>33328</v>
       </c>
       <c r="I3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
-        <f>E4-$Q$2</f>
+        <f>D4-$Q$2</f>
         <v>9360</v>
       </c>
       <c r="B4" s="1" t="str">
@@ -492,38 +511,178 @@
         <v>116224</v>
       </c>
       <c r="D4">
+        <v>33360</v>
+      </c>
+      <c r="E4">
         <f>C4-C3</f>
         <v>-1024</v>
       </c>
-      <c r="E4">
-        <v>33360</v>
-      </c>
-      <c r="F4" s="2">
-        <f>E4-E3</f>
+      <c r="F4">
+        <f>D4-D3</f>
         <v>32</v>
       </c>
       <c r="G4">
-        <f>$E$3-E4</f>
+        <f>$D$3-D4</f>
         <v>-32</v>
       </c>
       <c r="H4">
-        <f>$Q$2-E4</f>
+        <f>$Q$2-D4</f>
         <v>-9360</v>
       </c>
       <c r="I4" t="s">
-        <v>5</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>116736</v>
+      </c>
+      <c r="D5">
+        <v>33396</v>
+      </c>
+      <c r="E5">
+        <f>C5-C4</f>
+        <v>512</v>
+      </c>
+      <c r="F5">
+        <f>D5-D4</f>
+        <v>36</v>
+      </c>
+      <c r="G5">
+        <f>$D$3-D5</f>
+        <v>-68</v>
+      </c>
+      <c r="H5">
+        <f>$Q$2-D5</f>
+        <v>-9396</v>
+      </c>
+      <c r="I5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C6">
+        <v>115200</v>
+      </c>
+      <c r="D6">
+        <v>33188</v>
+      </c>
+      <c r="E6">
+        <f>C6-C5</f>
+        <v>-1536</v>
+      </c>
+      <c r="F6">
+        <f>D6-D5</f>
+        <v>-208</v>
+      </c>
+      <c r="G6">
+        <f>$D$3-D6</f>
+        <v>140</v>
+      </c>
+      <c r="H6">
+        <f>$Q$2-D6</f>
+        <v>-9188</v>
+      </c>
+      <c r="I6" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C42FA46-C395-40D3-849E-85E8997FBDEF}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>69705</v>
+      </c>
+      <c r="C2">
+        <v>12623</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>68052</v>
+      </c>
+      <c r="C3">
+        <v>12400</v>
+      </c>
+      <c r="D3">
+        <f>B3-$B$2</f>
+        <v>-1653</v>
+      </c>
+      <c r="E3">
+        <f>C3-$C$2</f>
+        <v>-223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>69540</v>
+      </c>
+      <c r="C4">
+        <v>12600</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:D5" si="0">B4-$B$2</f>
+        <v>-165</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E5" si="1">C4-$C$2</f>
+        <v>-23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <v>67887</v>
+      </c>
+      <c r="C5">
+        <v>12385</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>-1818</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>-238</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#185 graph processing simplified greatly
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706EE84C-66AB-4422-A26D-B8FB4C52FBF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49D9CBC-E38E-48FB-9335-C9783B095CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11070" yWindow="1260" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="11010" yWindow="900" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>target</t>
   </si>
@@ -80,6 +80,87 @@
   </si>
   <si>
     <t>with oneshot song payload</t>
+  </si>
+  <si>
+    <t>device sizes</t>
+  </si>
+  <si>
+    <t>no devices (only song data + player + wavwriter + overhead)</t>
+  </si>
+  <si>
+    <t>+eq only</t>
+  </si>
+  <si>
+    <t>+space only</t>
+  </si>
+  <si>
+    <t>+mbc only</t>
+  </si>
+  <si>
+    <t>+gigasynth only</t>
+  </si>
+  <si>
+    <t>from base</t>
+  </si>
+  <si>
+    <t>+eq, space, mbc</t>
+  </si>
+  <si>
+    <t>so, about 3kb is shared code between fx. 2kb is specific to the 3 effects</t>
+  </si>
+  <si>
+    <t>+gigasynth + eq</t>
+  </si>
+  <si>
+    <t>gigasynth+space</t>
+  </si>
+  <si>
+    <t>so EQ adds 368 bytes from gigasynth</t>
+  </si>
+  <si>
+    <t>wow space adds 1,2kb how??</t>
+  </si>
+  <si>
+    <t>gigasynth+space + eq</t>
+  </si>
+  <si>
+    <t>eq continues to show about 350 bytes of specific code.</t>
+  </si>
+  <si>
+    <t>gigasynth + mbc</t>
+  </si>
+  <si>
+    <t>gigasynth + mbc + space</t>
+  </si>
+  <si>
+    <t>so mbc seems to add 1,7kb</t>
+  </si>
+  <si>
+    <t>here space is showing 1kb more than mbc.</t>
+  </si>
+  <si>
+    <t>conclusion:</t>
+  </si>
+  <si>
+    <t>gigasynth itself is like 12kb of code.</t>
+  </si>
+  <si>
+    <t>eq is tiny because it's just filters used by gigasynth, about 350 bytes</t>
+  </si>
+  <si>
+    <t>space and mbc are about 1.5kb each</t>
+  </si>
+  <si>
+    <t>plan: monolithic effect device first, then make a budget for gigasynth</t>
+  </si>
+  <si>
+    <t>new graph runner: serialization additions, reading track flag</t>
+  </si>
+  <si>
+    <t>stripping out graph runner basically entirely</t>
+  </si>
+  <si>
+    <t>new graph runner working</t>
   </si>
 </sst>
 </file>
@@ -122,9 +203,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -439,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -514,11 +596,11 @@
         <v>33360</v>
       </c>
       <c r="E4">
-        <f>C4-C3</f>
+        <f t="shared" ref="E4:F6" si="1">C4-C3</f>
         <v>-1024</v>
       </c>
       <c r="F4">
-        <f>D4-D3</f>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="G4">
@@ -541,11 +623,11 @@
         <v>33396</v>
       </c>
       <c r="E5">
-        <f>C5-C4</f>
+        <f t="shared" si="1"/>
         <v>512</v>
       </c>
       <c r="F5">
-        <f>D5-D4</f>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="G5">
@@ -568,11 +650,11 @@
         <v>33188</v>
       </c>
       <c r="E6">
-        <f>C6-C5</f>
+        <f t="shared" si="1"/>
         <v>-1536</v>
       </c>
       <c r="F6">
-        <f>D6-D5</f>
+        <f t="shared" si="1"/>
         <v>-208</v>
       </c>
       <c r="G6">
@@ -585,6 +667,87 @@
       </c>
       <c r="I6" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>115200</v>
+      </c>
+      <c r="D7">
+        <v>33196</v>
+      </c>
+      <c r="E7">
+        <f t="shared" ref="E7" si="2">C7-C6</f>
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <f t="shared" ref="F7" si="3">D7-D6</f>
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <f>$D$3-D7</f>
+        <v>132</v>
+      </c>
+      <c r="H7">
+        <f>$Q$2-D7</f>
+        <v>-9196</v>
+      </c>
+      <c r="I7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>114176</v>
+      </c>
+      <c r="D8">
+        <v>32696</v>
+      </c>
+      <c r="E8">
+        <f t="shared" ref="E8" si="4">C8-C7</f>
+        <v>-1024</v>
+      </c>
+      <c r="F8">
+        <f t="shared" ref="F8" si="5">D8-D7</f>
+        <v>-500</v>
+      </c>
+      <c r="G8">
+        <f>$D$3-D8</f>
+        <v>632</v>
+      </c>
+      <c r="H8">
+        <f>$Q$2-D8</f>
+        <v>-8696</v>
+      </c>
+      <c r="I8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <v>114176</v>
+      </c>
+      <c r="D9">
+        <v>32792</v>
+      </c>
+      <c r="E9">
+        <f t="shared" ref="E9" si="6">C9-C8</f>
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <f t="shared" ref="F9" si="7">D9-D8</f>
+        <v>96</v>
+      </c>
+      <c r="G9">
+        <f>$D$3-D9</f>
+        <v>536</v>
+      </c>
+      <c r="H9">
+        <f>$Q$2-D9</f>
+        <v>-8792</v>
+      </c>
+      <c r="I9" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -595,15 +758,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C42FA46-C395-40D3-849E-85E8997FBDEF}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -614,7 +777,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -625,7 +788,7 @@
         <v>12623</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -644,7 +807,7 @@
         <v>-223</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -663,7 +826,7 @@
         <v>-23</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -680,6 +843,205 @@
       <c r="E5">
         <f t="shared" si="1"/>
         <v>-238</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10">
+        <v>18448</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>20936</v>
+      </c>
+      <c r="D11">
+        <f>C11-$C$10</f>
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12">
+        <v>21228</v>
+      </c>
+      <c r="D12">
+        <f t="shared" ref="D12:D20" si="2">C12-$C$10</f>
+        <v>2780</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13">
+        <v>21924</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="2"/>
+        <v>3476</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14">
+        <v>24008</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>5560</v>
+      </c>
+      <c r="F14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15">
+        <v>30048</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="2"/>
+        <v>11600</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16">
+        <v>30416</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="2"/>
+        <v>11968</v>
+      </c>
+      <c r="E16">
+        <f>C16-C15</f>
+        <v>368</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17">
+        <v>31292</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="2"/>
+        <v>12844</v>
+      </c>
+      <c r="E17">
+        <f>C17-C15</f>
+        <v>1244</v>
+      </c>
+      <c r="F17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18">
+        <v>31629</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="2"/>
+        <v>13181</v>
+      </c>
+      <c r="E18">
+        <f>C18-C17</f>
+        <v>337</v>
+      </c>
+      <c r="F18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19">
+        <v>31840</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="2"/>
+        <v>13392</v>
+      </c>
+      <c r="E19">
+        <f>C19-C15</f>
+        <v>1792</v>
+      </c>
+      <c r="F19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20">
+        <v>32868</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="2"/>
+        <v>14420</v>
+      </c>
+      <c r="E20">
+        <f>C19-C20</f>
+        <v>-1028</v>
+      </c>
+      <c r="F20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#184 removing filter circuit / slope, supporting ONLY single biquad + vanilla onepole
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89035D9-1136-4188-8C07-3C4DFE4B488F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759F54BA-5DC4-4BF6-860E-56A9F107592B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11010" yWindow="900" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="10785" yWindow="3030" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>target</t>
   </si>
@@ -167,6 +167,12 @@
   </si>
   <si>
     <t>this is the player, wav writer, graph runner overhead</t>
+  </si>
+  <si>
+    <t>maj7comp instead of mbc</t>
+  </si>
+  <si>
+    <t>removing selectable filter models &amp; slopes, using vanilla onepole</t>
   </si>
 </sst>
 </file>
@@ -527,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -592,8 +598,8 @@
         <v>9360</v>
       </c>
       <c r="B4" s="1" t="str">
-        <f t="shared" ref="B4" si="0">REPT("#",A4*100/MAX(A:A))</f>
-        <v>####################################################################################################</v>
+        <f>REPT("#",A4*100/MAX(A:A))</f>
+        <v>###################################################################################################</v>
       </c>
       <c r="C4">
         <v>116224</v>
@@ -602,19 +608,19 @@
         <v>33360</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E4:F6" si="1">C4-C3</f>
+        <f t="shared" ref="E4:F6" si="0">C4-C3</f>
         <v>-1024</v>
       </c>
       <c r="F4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="G4">
-        <f>$D$3-D4</f>
+        <f t="shared" ref="G4:G11" si="1">$D$3-D4</f>
         <v>-32</v>
       </c>
       <c r="H4">
-        <f>$Q$2-D4</f>
+        <f t="shared" ref="H4:H11" si="2">$Q$2-D4</f>
         <v>-9360</v>
       </c>
       <c r="I4" t="s">
@@ -622,6 +628,14 @@
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <f t="shared" ref="A5:A11" si="3">D5-$Q$2</f>
+        <v>9396</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <f t="shared" ref="B5:B11" si="4">REPT("#",A5*100/MAX(A:A))</f>
+        <v>####################################################################################################</v>
+      </c>
       <c r="C5">
         <v>116736</v>
       </c>
@@ -629,19 +643,19 @@
         <v>33396</v>
       </c>
       <c r="E5">
+        <f t="shared" si="0"/>
+        <v>512</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="G5">
         <f t="shared" si="1"/>
-        <v>512</v>
-      </c>
-      <c r="F5">
-        <f t="shared" si="1"/>
-        <v>36</v>
-      </c>
-      <c r="G5">
-        <f>$D$3-D5</f>
         <v>-68</v>
       </c>
       <c r="H5">
-        <f>$Q$2-D5</f>
+        <f t="shared" si="2"/>
         <v>-9396</v>
       </c>
       <c r="I5" t="s">
@@ -649,6 +663,14 @@
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <f t="shared" si="3"/>
+        <v>9188</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>#################################################################################################</v>
+      </c>
       <c r="C6">
         <v>115200</v>
       </c>
@@ -656,19 +678,19 @@
         <v>33188</v>
       </c>
       <c r="E6">
+        <f t="shared" si="0"/>
+        <v>-1536</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>-208</v>
+      </c>
+      <c r="G6">
         <f t="shared" si="1"/>
-        <v>-1536</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="1"/>
-        <v>-208</v>
-      </c>
-      <c r="G6">
-        <f>$D$3-D6</f>
         <v>140</v>
       </c>
       <c r="H6">
-        <f>$Q$2-D6</f>
+        <f t="shared" si="2"/>
         <v>-9188</v>
       </c>
       <c r="I6" t="s">
@@ -676,6 +698,14 @@
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <f t="shared" si="3"/>
+        <v>9196</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>#################################################################################################</v>
+      </c>
       <c r="C7">
         <v>115200</v>
       </c>
@@ -683,19 +713,19 @@
         <v>33196</v>
       </c>
       <c r="E7">
-        <f t="shared" ref="E7" si="2">C7-C6</f>
+        <f t="shared" ref="E7" si="5">C7-C6</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f t="shared" ref="F7" si="3">D7-D6</f>
+        <f t="shared" ref="F7" si="6">D7-D6</f>
         <v>8</v>
       </c>
       <c r="G7">
-        <f>$D$3-D7</f>
+        <f t="shared" si="1"/>
         <v>132</v>
       </c>
       <c r="H7">
-        <f>$Q$2-D7</f>
+        <f t="shared" si="2"/>
         <v>-9196</v>
       </c>
       <c r="I7" t="s">
@@ -703,6 +733,14 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <f t="shared" si="3"/>
+        <v>8696</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>############################################################################################</v>
+      </c>
       <c r="C8">
         <v>114176</v>
       </c>
@@ -710,19 +748,19 @@
         <v>32696</v>
       </c>
       <c r="E8">
-        <f t="shared" ref="E8" si="4">C8-C7</f>
+        <f t="shared" ref="E8" si="7">C8-C7</f>
         <v>-1024</v>
       </c>
       <c r="F8">
-        <f t="shared" ref="F8" si="5">D8-D7</f>
+        <f t="shared" ref="F8" si="8">D8-D7</f>
         <v>-500</v>
       </c>
       <c r="G8">
-        <f>$D$3-D8</f>
+        <f t="shared" si="1"/>
         <v>632</v>
       </c>
       <c r="H8">
-        <f>$Q$2-D8</f>
+        <f t="shared" si="2"/>
         <v>-8696</v>
       </c>
       <c r="I8" t="s">
@@ -730,6 +768,14 @@
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <f t="shared" si="3"/>
+        <v>8792</v>
+      </c>
+      <c r="B9" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>#############################################################################################</v>
+      </c>
       <c r="C9">
         <v>114176</v>
       </c>
@@ -737,23 +783,93 @@
         <v>32792</v>
       </c>
       <c r="E9">
-        <f t="shared" ref="E9" si="6">C9-C8</f>
+        <f t="shared" ref="E9" si="9">C9-C8</f>
         <v>0</v>
       </c>
       <c r="F9">
-        <f t="shared" ref="F9" si="7">D9-D8</f>
+        <f t="shared" ref="F9" si="10">D9-D8</f>
         <v>96</v>
       </c>
       <c r="G9">
-        <f>$D$3-D9</f>
+        <f t="shared" si="1"/>
         <v>536</v>
       </c>
       <c r="H9">
-        <f>$Q$2-D9</f>
+        <f t="shared" si="2"/>
         <v>-8792</v>
       </c>
       <c r="I9" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <f t="shared" si="3"/>
+        <v>7744</v>
+      </c>
+      <c r="B10" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>##################################################################################</v>
+      </c>
+      <c r="C10">
+        <v>111104</v>
+      </c>
+      <c r="D10">
+        <v>31744</v>
+      </c>
+      <c r="E10">
+        <f t="shared" ref="E10" si="11">C10-C9</f>
+        <v>-3072</v>
+      </c>
+      <c r="F10">
+        <f t="shared" ref="F10" si="12">D10-D9</f>
+        <v>-1048</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="1"/>
+        <v>1584</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="2"/>
+        <v>-7744</v>
+      </c>
+      <c r="I10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <f t="shared" si="3"/>
+        <v>7124</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>###########################################################################</v>
+      </c>
+      <c r="C11">
+        <v>109568</v>
+      </c>
+      <c r="D11">
+        <v>31124</v>
+      </c>
+      <c r="E11">
+        <f t="shared" ref="E11" si="13">C11-C10</f>
+        <v>-1536</v>
+      </c>
+      <c r="F11">
+        <f t="shared" ref="F11" si="14">D11-D10</f>
+        <v>-620</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="1"/>
+        <v>2204</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="2"/>
+        <v>-7124</v>
+      </c>
+      <c r="I11" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#184 adding softclip to comp
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759F54BA-5DC4-4BF6-860E-56A9F107592B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B5470B-6363-4313-8D31-EC416C1CC666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10785" yWindow="3030" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>target</t>
   </si>
@@ -173,6 +173,12 @@
   </si>
   <si>
     <t>removing selectable filter models &amp; slopes, using vanilla onepole</t>
+  </si>
+  <si>
+    <t>removing LP and Q from sidechain</t>
+  </si>
+  <si>
+    <t>adding in sineclipper to comp</t>
   </si>
 </sst>
 </file>
@@ -533,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -616,11 +622,11 @@
         <v>32</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4:G11" si="1">$D$3-D4</f>
+        <f t="shared" ref="G4:G13" si="1">$D$3-D4</f>
         <v>-32</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H4:H11" si="2">$Q$2-D4</f>
+        <f t="shared" ref="H4:H13" si="2">$Q$2-D4</f>
         <v>-9360</v>
       </c>
       <c r="I4" t="s">
@@ -629,11 +635,11 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
-        <f t="shared" ref="A5:A11" si="3">D5-$Q$2</f>
+        <f t="shared" ref="A5:A13" si="3">D5-$Q$2</f>
         <v>9396</v>
       </c>
       <c r="B5" s="1" t="str">
-        <f t="shared" ref="B5:B11" si="4">REPT("#",A5*100/MAX(A:A))</f>
+        <f t="shared" ref="B5:B13" si="4">REPT("#",A5*100/MAX(A:A))</f>
         <v>####################################################################################################</v>
       </c>
       <c r="C5">
@@ -870,6 +876,76 @@
       </c>
       <c r="I11" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <f t="shared" si="3"/>
+        <v>7104</v>
+      </c>
+      <c r="B12" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>###########################################################################</v>
+      </c>
+      <c r="C12">
+        <v>109568</v>
+      </c>
+      <c r="D12">
+        <v>31104</v>
+      </c>
+      <c r="E12">
+        <f t="shared" ref="E12" si="15">C12-C11</f>
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <f t="shared" ref="F12" si="16">D12-D11</f>
+        <v>-20</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="1"/>
+        <v>2224</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="2"/>
+        <v>-7104</v>
+      </c>
+      <c r="I12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <f t="shared" si="3"/>
+        <v>7108</v>
+      </c>
+      <c r="B13" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>###########################################################################</v>
+      </c>
+      <c r="C13">
+        <v>109568</v>
+      </c>
+      <c r="D13">
+        <v>31108</v>
+      </c>
+      <c r="E13">
+        <f t="shared" ref="E13" si="17">C13-C12</f>
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13" si="18">D13-D12</f>
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="1"/>
+        <v>2220</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="2"/>
+        <v>-7108</v>
+      </c>
+      <c r="I13" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#184 removing cc, pb, sustain support
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B5470B-6363-4313-8D31-EC416C1CC666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06F3F64-3205-4CDC-992B-E5AE7FB4B860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10785" yWindow="3030" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>target</t>
   </si>
@@ -179,6 +179,18 @@
   </si>
   <si>
     <t>adding in sineclipper to comp</t>
+  </si>
+  <si>
+    <t>remove output stream from comp</t>
+  </si>
+  <si>
+    <t>duplicating EQ defaults instead of custom per band</t>
+  </si>
+  <si>
+    <t>remove 2nd filter from gigasynth</t>
+  </si>
+  <si>
+    <t>no CC, pitchbend, sustain pedal support</t>
   </si>
 </sst>
 </file>
@@ -539,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -622,11 +634,11 @@
         <v>32</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4:G13" si="1">$D$3-D4</f>
+        <f t="shared" ref="G4:G17" si="1">$D$3-D4</f>
         <v>-32</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H4:H13" si="2">$Q$2-D4</f>
+        <f t="shared" ref="H4:H17" si="2">$Q$2-D4</f>
         <v>-9360</v>
       </c>
       <c r="I4" t="s">
@@ -635,11 +647,11 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
-        <f t="shared" ref="A5:A13" si="3">D5-$Q$2</f>
+        <f t="shared" ref="A5:A17" si="3">D5-$Q$2</f>
         <v>9396</v>
       </c>
       <c r="B5" s="1" t="str">
-        <f t="shared" ref="B5:B13" si="4">REPT("#",A5*100/MAX(A:A))</f>
+        <f t="shared" ref="B5:B17" si="4">REPT("#",A5*100/MAX(A:A))</f>
         <v>####################################################################################################</v>
       </c>
       <c r="C5">
@@ -946,6 +958,146 @@
       </c>
       <c r="I13" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <f t="shared" si="3"/>
+        <v>7092</v>
+      </c>
+      <c r="B14" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>###########################################################################</v>
+      </c>
+      <c r="C14">
+        <v>109568</v>
+      </c>
+      <c r="D14">
+        <v>31092</v>
+      </c>
+      <c r="E14">
+        <f t="shared" ref="E14" si="19">C14-C13</f>
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <f t="shared" ref="F14" si="20">D14-D13</f>
+        <v>-16</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>2236</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>-7092</v>
+      </c>
+      <c r="I14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <f t="shared" si="3"/>
+        <v>7076</v>
+      </c>
+      <c r="B15" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>###########################################################################</v>
+      </c>
+      <c r="C15">
+        <v>109568</v>
+      </c>
+      <c r="D15">
+        <v>31076</v>
+      </c>
+      <c r="E15">
+        <f t="shared" ref="E15" si="21">C15-C14</f>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" ref="F15" si="22">D15-D14</f>
+        <v>-16</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="1"/>
+        <v>2252</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="2"/>
+        <v>-7076</v>
+      </c>
+      <c r="I15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <f t="shared" si="3"/>
+        <v>7016</v>
+      </c>
+      <c r="B16" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>##########################################################################</v>
+      </c>
+      <c r="C16">
+        <v>108544</v>
+      </c>
+      <c r="D16">
+        <v>31016</v>
+      </c>
+      <c r="E16">
+        <f t="shared" ref="E16" si="23">C16-C15</f>
+        <v>-1024</v>
+      </c>
+      <c r="F16">
+        <f t="shared" ref="F16" si="24">D16-D15</f>
+        <v>-60</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="1"/>
+        <v>2312</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="2"/>
+        <v>-7016</v>
+      </c>
+      <c r="I16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <f t="shared" si="3"/>
+        <v>6868</v>
+      </c>
+      <c r="B17" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>#########################################################################</v>
+      </c>
+      <c r="C17">
+        <v>108544</v>
+      </c>
+      <c r="D17">
+        <v>30868</v>
+      </c>
+      <c r="E17">
+        <f t="shared" ref="E17" si="25">C17-C16</f>
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <f t="shared" ref="F17" si="26">D17-D16</f>
+        <v>-148</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="1"/>
+        <v>2460</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="2"/>
+        <v>-6868</v>
+      </c>
+      <c r="I17" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#184 reducing macro count to 4, removing LFO time basis
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06F3F64-3205-4CDC-992B-E5AE7FB4B860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175AF008-AAC1-4E9B-B338-2881E6C9484A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10785" yWindow="3030" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="11010" yWindow="900" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>target</t>
   </si>
@@ -191,6 +191,21 @@
   </si>
   <si>
     <t>no CC, pitchbend, sustain pedal support</t>
+  </si>
+  <si>
+    <t>more cleanups removing/unifying filters</t>
+  </si>
+  <si>
+    <t>removing folded sine, evolving grain osc</t>
+  </si>
+  <si>
+    <t>remove polyblep from S&amp;H noise</t>
+  </si>
+  <si>
+    <t>remove whitenoise (use SH)</t>
+  </si>
+  <si>
+    <t>remove shapes -- only naïve trap. Removing pulse3 while I'm at it.</t>
   </si>
 </sst>
 </file>
@@ -551,7 +566,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -634,11 +649,11 @@
         <v>32</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4:G17" si="1">$D$3-D4</f>
+        <f t="shared" ref="G4:G23" si="1">$D$3-D4</f>
         <v>-32</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H4:H17" si="2">$Q$2-D4</f>
+        <f t="shared" ref="H4:H23" si="2">$Q$2-D4</f>
         <v>-9360</v>
       </c>
       <c r="I4" t="s">
@@ -647,11 +662,11 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
-        <f t="shared" ref="A5:A17" si="3">D5-$Q$2</f>
+        <f t="shared" ref="A5:A23" si="3">D5-$Q$2</f>
         <v>9396</v>
       </c>
       <c r="B5" s="1" t="str">
-        <f t="shared" ref="B5:B17" si="4">REPT("#",A5*100/MAX(A:A))</f>
+        <f t="shared" ref="B5:B23" si="4">REPT("#",A5*100/MAX(A:A))</f>
         <v>####################################################################################################</v>
       </c>
       <c r="C5">
@@ -1098,6 +1113,191 @@
       </c>
       <c r="I17" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <f t="shared" si="3"/>
+        <v>6756</v>
+      </c>
+      <c r="B18" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>#######################################################################</v>
+      </c>
+      <c r="C18">
+        <v>108544</v>
+      </c>
+      <c r="D18">
+        <v>30756</v>
+      </c>
+      <c r="E18">
+        <f t="shared" ref="E18" si="27">C18-C17</f>
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <f t="shared" ref="F18" si="28">D18-D17</f>
+        <v>-112</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="1"/>
+        <v>2572</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="2"/>
+        <v>-6756</v>
+      </c>
+      <c r="I18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <f t="shared" si="3"/>
+        <v>6404</v>
+      </c>
+      <c r="B19" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>####################################################################</v>
+      </c>
+      <c r="C19">
+        <v>107008</v>
+      </c>
+      <c r="D19">
+        <v>30404</v>
+      </c>
+      <c r="E19">
+        <f t="shared" ref="E19" si="29">C19-C18</f>
+        <v>-1536</v>
+      </c>
+      <c r="F19">
+        <f t="shared" ref="F19" si="30">D19-D18</f>
+        <v>-352</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="1"/>
+        <v>2924</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>-6404</v>
+      </c>
+      <c r="I19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <f t="shared" si="3"/>
+        <v>6344</v>
+      </c>
+      <c r="B20" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>###################################################################</v>
+      </c>
+      <c r="C20">
+        <v>107008</v>
+      </c>
+      <c r="D20">
+        <v>30344</v>
+      </c>
+      <c r="E20">
+        <f t="shared" ref="E20" si="31">C20-C19</f>
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <f t="shared" ref="F20" si="32">D20-D19</f>
+        <v>-60</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="1"/>
+        <v>2984</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="2"/>
+        <v>-6344</v>
+      </c>
+      <c r="I20" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <f t="shared" si="3"/>
+        <v>6268</v>
+      </c>
+      <c r="B21" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>##################################################################</v>
+      </c>
+      <c r="C21">
+        <v>106496</v>
+      </c>
+      <c r="D21">
+        <v>30268</v>
+      </c>
+      <c r="E21">
+        <f t="shared" ref="E21" si="33">C21-C20</f>
+        <v>-512</v>
+      </c>
+      <c r="F21">
+        <f t="shared" ref="F21" si="34">D21-D20</f>
+        <v>-76</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="1"/>
+        <v>3060</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="2"/>
+        <v>-6268</v>
+      </c>
+      <c r="I21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <f t="shared" si="3"/>
+        <v>5612</v>
+      </c>
+      <c r="B22" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>###########################################################</v>
+      </c>
+      <c r="C22">
+        <v>104960</v>
+      </c>
+      <c r="D22">
+        <v>29612</v>
+      </c>
+      <c r="E22">
+        <f t="shared" ref="E22" si="35">C22-C21</f>
+        <v>-1536</v>
+      </c>
+      <c r="F22">
+        <f t="shared" ref="F22" si="36">D22-D21</f>
+        <v>-656</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="1"/>
+        <v>3716</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="2"/>
+        <v>-5612</v>
+      </c>
+      <c r="I22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <f t="shared" si="3"/>
+        <v>-24000</v>
+      </c>
+      <c r="B23" s="1" t="e">
+        <f t="shared" si="4"/>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding soft clip ctrls to comp
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175AF008-AAC1-4E9B-B338-2881E6C9484A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D1DF0D-A76B-46E9-A19A-97983A1DDD8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11010" yWindow="900" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>target</t>
   </si>
@@ -206,6 +206,24 @@
   </si>
   <si>
     <t>remove shapes -- only naïve trap. Removing pulse3 while I'm at it.</t>
+  </si>
+  <si>
+    <t>macro count -&gt; 4</t>
+  </si>
+  <si>
+    <t>remove time basis from LFO</t>
+  </si>
+  <si>
+    <t>remove mod aux</t>
+  </si>
+  <si>
+    <t>remove mod curve support</t>
+  </si>
+  <si>
+    <t>remove osc compensation gain</t>
+  </si>
+  <si>
+    <t>remove sampler device entirely</t>
   </si>
 </sst>
 </file>
@@ -221,7 +239,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="4"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -250,8 +268,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,10 +584,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -611,7 +629,7 @@
         <f>D3-$Q$2</f>
         <v>9328</v>
       </c>
-      <c r="B3" s="1" t="str">
+      <c r="B3" s="2" t="str">
         <f>REPT("#",A3*100/MAX(A:A))</f>
         <v>###################################################################################################</v>
       </c>
@@ -630,7 +648,7 @@
         <f>D4-$Q$2</f>
         <v>9360</v>
       </c>
-      <c r="B4" s="1" t="str">
+      <c r="B4" s="2" t="str">
         <f>REPT("#",A4*100/MAX(A:A))</f>
         <v>###################################################################################################</v>
       </c>
@@ -649,11 +667,11 @@
         <v>32</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4:G23" si="1">$D$3-D4</f>
+        <f t="shared" ref="G4:G26" si="1">$D$3-D4</f>
         <v>-32</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H4:H23" si="2">$Q$2-D4</f>
+        <f t="shared" ref="H4:H26" si="2">$Q$2-D4</f>
         <v>-9360</v>
       </c>
       <c r="I4" t="s">
@@ -662,11 +680,11 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
-        <f t="shared" ref="A5:A23" si="3">D5-$Q$2</f>
+        <f t="shared" ref="A5:A26" si="3">D5-$Q$2</f>
         <v>9396</v>
       </c>
-      <c r="B5" s="1" t="str">
-        <f t="shared" ref="B5:B23" si="4">REPT("#",A5*100/MAX(A:A))</f>
+      <c r="B5" s="2" t="str">
+        <f t="shared" ref="B5:B26" si="4">REPT("#",A5*100/MAX(A:A))</f>
         <v>####################################################################################################</v>
       </c>
       <c r="C5">
@@ -700,7 +718,7 @@
         <f t="shared" si="3"/>
         <v>9188</v>
       </c>
-      <c r="B6" s="1" t="str">
+      <c r="B6" s="2" t="str">
         <f t="shared" si="4"/>
         <v>#################################################################################################</v>
       </c>
@@ -735,7 +753,7 @@
         <f t="shared" si="3"/>
         <v>9196</v>
       </c>
-      <c r="B7" s="1" t="str">
+      <c r="B7" s="2" t="str">
         <f t="shared" si="4"/>
         <v>#################################################################################################</v>
       </c>
@@ -770,7 +788,7 @@
         <f t="shared" si="3"/>
         <v>8696</v>
       </c>
-      <c r="B8" s="1" t="str">
+      <c r="B8" s="2" t="str">
         <f t="shared" si="4"/>
         <v>############################################################################################</v>
       </c>
@@ -805,7 +823,7 @@
         <f t="shared" si="3"/>
         <v>8792</v>
       </c>
-      <c r="B9" s="1" t="str">
+      <c r="B9" s="2" t="str">
         <f t="shared" si="4"/>
         <v>#############################################################################################</v>
       </c>
@@ -840,7 +858,7 @@
         <f t="shared" si="3"/>
         <v>7744</v>
       </c>
-      <c r="B10" s="1" t="str">
+      <c r="B10" s="2" t="str">
         <f t="shared" si="4"/>
         <v>##################################################################################</v>
       </c>
@@ -875,7 +893,7 @@
         <f t="shared" si="3"/>
         <v>7124</v>
       </c>
-      <c r="B11" s="1" t="str">
+      <c r="B11" s="2" t="str">
         <f t="shared" si="4"/>
         <v>###########################################################################</v>
       </c>
@@ -910,7 +928,7 @@
         <f t="shared" si="3"/>
         <v>7104</v>
       </c>
-      <c r="B12" s="1" t="str">
+      <c r="B12" s="2" t="str">
         <f t="shared" si="4"/>
         <v>###########################################################################</v>
       </c>
@@ -945,7 +963,7 @@
         <f t="shared" si="3"/>
         <v>7108</v>
       </c>
-      <c r="B13" s="1" t="str">
+      <c r="B13" s="2" t="str">
         <f t="shared" si="4"/>
         <v>###########################################################################</v>
       </c>
@@ -980,7 +998,7 @@
         <f t="shared" si="3"/>
         <v>7092</v>
       </c>
-      <c r="B14" s="1" t="str">
+      <c r="B14" s="2" t="str">
         <f t="shared" si="4"/>
         <v>###########################################################################</v>
       </c>
@@ -1015,7 +1033,7 @@
         <f t="shared" si="3"/>
         <v>7076</v>
       </c>
-      <c r="B15" s="1" t="str">
+      <c r="B15" s="2" t="str">
         <f t="shared" si="4"/>
         <v>###########################################################################</v>
       </c>
@@ -1050,7 +1068,7 @@
         <f t="shared" si="3"/>
         <v>7016</v>
       </c>
-      <c r="B16" s="1" t="str">
+      <c r="B16" s="2" t="str">
         <f t="shared" si="4"/>
         <v>##########################################################################</v>
       </c>
@@ -1085,7 +1103,7 @@
         <f t="shared" si="3"/>
         <v>6868</v>
       </c>
-      <c r="B17" s="1" t="str">
+      <c r="B17" s="2" t="str">
         <f t="shared" si="4"/>
         <v>#########################################################################</v>
       </c>
@@ -1120,7 +1138,7 @@
         <f t="shared" si="3"/>
         <v>6756</v>
       </c>
-      <c r="B18" s="1" t="str">
+      <c r="B18" s="2" t="str">
         <f t="shared" si="4"/>
         <v>#######################################################################</v>
       </c>
@@ -1155,7 +1173,7 @@
         <f t="shared" si="3"/>
         <v>6404</v>
       </c>
-      <c r="B19" s="1" t="str">
+      <c r="B19" s="2" t="str">
         <f t="shared" si="4"/>
         <v>####################################################################</v>
       </c>
@@ -1190,7 +1208,7 @@
         <f t="shared" si="3"/>
         <v>6344</v>
       </c>
-      <c r="B20" s="1" t="str">
+      <c r="B20" s="2" t="str">
         <f t="shared" si="4"/>
         <v>###################################################################</v>
       </c>
@@ -1225,7 +1243,7 @@
         <f t="shared" si="3"/>
         <v>6268</v>
       </c>
-      <c r="B21" s="1" t="str">
+      <c r="B21" s="2" t="str">
         <f t="shared" si="4"/>
         <v>##################################################################</v>
       </c>
@@ -1260,7 +1278,7 @@
         <f t="shared" si="3"/>
         <v>5612</v>
       </c>
-      <c r="B22" s="1" t="str">
+      <c r="B22" s="2" t="str">
         <f t="shared" si="4"/>
         <v>###########################################################</v>
       </c>
@@ -1293,11 +1311,211 @@
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="3"/>
-        <v>-24000</v>
-      </c>
-      <c r="B23" s="1" t="e">
-        <f t="shared" si="4"/>
-        <v>#VALUE!</v>
+        <v>5608</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <f t="shared" si="4"/>
+        <v>###########################################################</v>
+      </c>
+      <c r="C23">
+        <v>104960</v>
+      </c>
+      <c r="D23">
+        <v>29608</v>
+      </c>
+      <c r="E23">
+        <f t="shared" ref="E23" si="37">C23-C22</f>
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <f t="shared" ref="F23" si="38">D23-D22</f>
+        <v>-4</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="1"/>
+        <v>3720</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="2"/>
+        <v>-5608</v>
+      </c>
+      <c r="I23" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <f t="shared" si="3"/>
+        <v>5496</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <f t="shared" si="4"/>
+        <v>##########################################################</v>
+      </c>
+      <c r="C24">
+        <v>104960</v>
+      </c>
+      <c r="D24">
+        <v>29496</v>
+      </c>
+      <c r="E24">
+        <f t="shared" ref="E24" si="39">C24-C23</f>
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <f t="shared" ref="F24" si="40">D24-D23</f>
+        <v>-112</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="1"/>
+        <v>3832</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="2"/>
+        <v>-5496</v>
+      </c>
+      <c r="I24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <f t="shared" si="3"/>
+        <v>5420</v>
+      </c>
+      <c r="B25" s="2" t="str">
+        <f t="shared" si="4"/>
+        <v>#########################################################</v>
+      </c>
+      <c r="C25">
+        <v>104448</v>
+      </c>
+      <c r="D25">
+        <v>29420</v>
+      </c>
+      <c r="E25">
+        <f t="shared" ref="E25" si="41">C25-C24</f>
+        <v>-512</v>
+      </c>
+      <c r="F25">
+        <f t="shared" ref="F25" si="42">D25-D24</f>
+        <v>-76</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="1"/>
+        <v>3908</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="2"/>
+        <v>-5420</v>
+      </c>
+      <c r="I25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <f t="shared" si="3"/>
+        <v>5404</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <f t="shared" si="4"/>
+        <v>#########################################################</v>
+      </c>
+      <c r="C26">
+        <v>104448</v>
+      </c>
+      <c r="D26">
+        <v>29404</v>
+      </c>
+      <c r="E26">
+        <f t="shared" ref="E26" si="43">C26-C25</f>
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <f t="shared" ref="F26" si="44">D26-D25</f>
+        <v>-16</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="1"/>
+        <v>3924</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="2"/>
+        <v>-5404</v>
+      </c>
+      <c r="I26" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <f t="shared" ref="A27:A28" si="45">D27-$Q$2</f>
+        <v>5392</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <f t="shared" ref="B27:B28" si="46">REPT("#",A27*100/MAX(A:A))</f>
+        <v>#########################################################</v>
+      </c>
+      <c r="C27">
+        <v>104448</v>
+      </c>
+      <c r="D27">
+        <v>29392</v>
+      </c>
+      <c r="E27">
+        <f t="shared" ref="E27" si="47">C27-C26</f>
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <f t="shared" ref="F27" si="48">D27-D26</f>
+        <v>-12</v>
+      </c>
+      <c r="G27">
+        <f t="shared" ref="G27:G28" si="49">$D$3-D27</f>
+        <v>3936</v>
+      </c>
+      <c r="H27">
+        <f t="shared" ref="H27:H28" si="50">$Q$2-D27</f>
+        <v>-5392</v>
+      </c>
+      <c r="I27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <f t="shared" si="45"/>
+        <v>4276</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <f t="shared" si="46"/>
+        <v>#############################################</v>
+      </c>
+      <c r="C28">
+        <v>102400</v>
+      </c>
+      <c r="D28">
+        <v>28276</v>
+      </c>
+      <c r="E28">
+        <f t="shared" ref="E28" si="51">C28-C27</f>
+        <v>-2048</v>
+      </c>
+      <c r="F28">
+        <f t="shared" ref="F28" si="52">D28-D27</f>
+        <v>-1116</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="49"/>
+        <v>5052</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="50"/>
+        <v>-4276</v>
+      </c>
+      <c r="I28" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1412,7 +1630,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C11">
@@ -1424,7 +1642,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C12">
@@ -1436,7 +1654,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C13">
@@ -1448,7 +1666,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C14">
@@ -1463,7 +1681,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C15">
@@ -1475,7 +1693,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C16">
@@ -1494,7 +1712,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C17">
@@ -1513,7 +1731,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C18">
@@ -1532,7 +1750,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C19">
@@ -1551,7 +1769,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C20">

</xml_diff>

<commit_message>
optimized gm.dls parsing #187
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D1DF0D-A76B-46E9-A19A-97983A1DDD8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07BA776-F62B-492C-8A63-F554458DE5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11010" yWindow="900" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>target</t>
   </si>
@@ -224,6 +224,18 @@
   </si>
   <si>
     <t>remove sampler device entirely</t>
+  </si>
+  <si>
+    <t>re-introduce mod aux, but without curve</t>
+  </si>
+  <si>
+    <t>remove shelving filters</t>
+  </si>
+  <si>
+    <t>re-enabling samplers</t>
+  </si>
+  <si>
+    <t>optimizing gmdls parsing</t>
   </si>
 </sst>
 </file>
@@ -584,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="44.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -1450,11 +1462,11 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
-        <f t="shared" ref="A27:A28" si="45">D27-$Q$2</f>
+        <f t="shared" ref="A27:A32" si="45">D27-$Q$2</f>
         <v>5392</v>
       </c>
       <c r="B27" s="2" t="str">
-        <f t="shared" ref="B27:B28" si="46">REPT("#",A27*100/MAX(A:A))</f>
+        <f t="shared" ref="B27:B32" si="46">REPT("#",A27*100/MAX(A:A))</f>
         <v>#########################################################</v>
       </c>
       <c r="C27">
@@ -1472,11 +1484,11 @@
         <v>-12</v>
       </c>
       <c r="G27">
-        <f t="shared" ref="G27:G28" si="49">$D$3-D27</f>
+        <f t="shared" ref="G27:G32" si="49">$D$3-D27</f>
         <v>3936</v>
       </c>
       <c r="H27">
-        <f t="shared" ref="H27:H28" si="50">$Q$2-D27</f>
+        <f t="shared" ref="H27:H32" si="50">$Q$2-D27</f>
         <v>-5392</v>
       </c>
       <c r="I27" t="s">
@@ -1516,6 +1528,140 @@
       </c>
       <c r="I28" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <f t="shared" si="45"/>
+        <v>4356</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <f t="shared" si="46"/>
+        <v>##############################################</v>
+      </c>
+      <c r="C29">
+        <v>102400</v>
+      </c>
+      <c r="D29">
+        <v>28356</v>
+      </c>
+      <c r="E29">
+        <f t="shared" ref="E29" si="53">C29-C28</f>
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <f t="shared" ref="F29" si="54">D29-D28</f>
+        <v>80</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="49"/>
+        <v>4972</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="50"/>
+        <v>-4356</v>
+      </c>
+      <c r="I29" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <f t="shared" si="45"/>
+        <v>4276</v>
+      </c>
+      <c r="B30" s="2" t="str">
+        <f t="shared" si="46"/>
+        <v>#############################################</v>
+      </c>
+      <c r="C30">
+        <v>102400</v>
+      </c>
+      <c r="D30">
+        <v>28276</v>
+      </c>
+      <c r="E30">
+        <f t="shared" ref="E30" si="55">C30-C29</f>
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <f t="shared" ref="F30" si="56">D30-D29</f>
+        <v>-80</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="49"/>
+        <v>5052</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="50"/>
+        <v>-4276</v>
+      </c>
+      <c r="I30" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <f t="shared" si="45"/>
+        <v>5408</v>
+      </c>
+      <c r="B31" s="2" t="str">
+        <f t="shared" si="46"/>
+        <v>#########################################################</v>
+      </c>
+      <c r="D31">
+        <v>29408</v>
+      </c>
+      <c r="E31">
+        <f t="shared" ref="E31" si="57">C31-C30</f>
+        <v>-102400</v>
+      </c>
+      <c r="F31">
+        <f t="shared" ref="F31" si="58">D31-D30</f>
+        <v>1132</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="49"/>
+        <v>3920</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="50"/>
+        <v>-5408</v>
+      </c>
+      <c r="I31" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <f t="shared" si="45"/>
+        <v>5276</v>
+      </c>
+      <c r="B32" s="2" t="str">
+        <f t="shared" si="46"/>
+        <v>########################################################</v>
+      </c>
+      <c r="D32">
+        <v>29276</v>
+      </c>
+      <c r="E32">
+        <f t="shared" ref="E32" si="59">C32-C31</f>
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <f t="shared" ref="F32" si="60">D32-D31</f>
+        <v>-132</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="49"/>
+        <v>4052</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="50"/>
+        <v>-5276</v>
+      </c>
+      <c r="I32" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sampler loop mode is now boolean, removing pingpong, removing reverse playback #187
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07BA776-F62B-492C-8A63-F554458DE5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20F1E4D-7252-42B6-AB0B-EE34CE30778E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11010" yWindow="900" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t>target</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>optimizing gmdls parsing</t>
+  </si>
+  <si>
+    <t>no reverse or ping pong loop; loop enable is boolean</t>
   </si>
 </sst>
 </file>
@@ -596,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="44.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -1635,14 +1638,14 @@
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
         <f t="shared" si="45"/>
-        <v>5276</v>
+        <v>5360</v>
       </c>
       <c r="B32" s="2" t="str">
         <f t="shared" si="46"/>
-        <v>########################################################</v>
+        <v>#########################################################</v>
       </c>
       <c r="D32">
-        <v>29276</v>
+        <v>29360</v>
       </c>
       <c r="E32">
         <f t="shared" ref="E32" si="59">C32-C31</f>
@@ -1650,18 +1653,42 @@
       </c>
       <c r="F32">
         <f t="shared" ref="F32" si="60">D32-D31</f>
-        <v>-132</v>
+        <v>-48</v>
       </c>
       <c r="G32">
         <f t="shared" si="49"/>
-        <v>4052</v>
+        <v>3968</v>
       </c>
       <c r="H32">
         <f t="shared" si="50"/>
-        <v>-5276</v>
+        <v>-5360</v>
       </c>
       <c r="I32" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D33">
+        <v>29260</v>
+      </c>
+      <c r="E33">
+        <f t="shared" ref="E33" si="61">C33-C32</f>
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <f t="shared" ref="F33" si="62">D33-D32</f>
+        <v>-100</v>
+      </c>
+      <c r="G33">
+        <f t="shared" ref="G33" si="63">$D$3-D33</f>
+        <v>4068</v>
+      </c>
+      <c r="H33">
+        <f t="shared" ref="H33" si="64">$Q$2-D33</f>
+        <v>-5260</v>
+      </c>
+      <c r="I33" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
merging from master #187 a15ca1a10bf53e5d53f03a30f891cd6dcb3c24f6 - gmdls sample player now uses span
</commit_message>
<xml_diff>
--- a/sizework20260410.xlsx
+++ b/sizework20260410.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A84F9227-BB01-41A0-AAFD-AD356F8E26A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09426723-D54B-44D3-BC11-44120C852432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11010" yWindow="900" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>target</t>
   </si>
@@ -242,6 +242,9 @@
   </si>
   <si>
     <t>remove loop boundary mode, more tweaks</t>
+  </si>
+  <si>
+    <t>gmdls optimizations</t>
   </si>
 </sst>
 </file>
@@ -602,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="44.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -1744,6 +1747,41 @@
       </c>
       <c r="I34" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <f t="shared" ref="A35" si="71">D35-$Q$2</f>
+        <v>5132</v>
+      </c>
+      <c r="B35" s="2" t="str">
+        <f t="shared" ref="B35" si="72">REPT("#",A35*100/MAX(A:A))</f>
+        <v>######################################################</v>
+      </c>
+      <c r="C35">
+        <v>103936</v>
+      </c>
+      <c r="D35">
+        <v>29132</v>
+      </c>
+      <c r="E35">
+        <f t="shared" ref="E35" si="73">C35-C34</f>
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <f t="shared" ref="F35" si="74">D35-D34</f>
+        <v>-48</v>
+      </c>
+      <c r="G35">
+        <f t="shared" ref="G35" si="75">$D$3-D35</f>
+        <v>4196</v>
+      </c>
+      <c r="H35">
+        <f t="shared" ref="H35" si="76">$Q$2-D35</f>
+        <v>-5132</v>
+      </c>
+      <c r="I35" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>